<commit_message>
Work in progress - data analysis
</commit_message>
<xml_diff>
--- a/Data/port.xlsx
+++ b/Data/port.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ricca\PycharmProjects\FantaAnalisi\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ricca\Documents\0003_Fantanalisi\FantaAnalisi\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52246ED5-7E9C-4E80-A956-231F83F06ABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84214FBE-0300-42FA-814C-0D786AB2F23B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3792" yWindow="4008" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Griglia portieri fantacalcio" sheetId="1" r:id="rId1"/>
@@ -20,9 +20,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="23">
-  <si>
-    <t>Griglia Portieri Fantacalcio.it 2024/25</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="22">
+  <si>
+    <t>Griglia Portieri Fantacalcio.it 2025/26</t>
   </si>
   <si>
     <t>Ata</t>
@@ -37,7 +37,7 @@
     <t>Com</t>
   </si>
   <si>
-    <t>Emp</t>
+    <t>Cre</t>
   </si>
   <si>
     <t>Fio</t>
@@ -61,34 +61,31 @@
     <t>Mil</t>
   </si>
   <si>
-    <t>Mon</t>
-  </si>
-  <si>
     <t>Nap</t>
   </si>
   <si>
     <t>Par</t>
   </si>
   <si>
+    <t>Pis</t>
+  </si>
+  <si>
     <t>Rom</t>
   </si>
   <si>
+    <t>Sas</t>
+  </si>
+  <si>
     <t>Tor</t>
   </si>
   <si>
     <t>Udi</t>
   </si>
   <si>
-    <t>Ven</t>
-  </si>
-  <si>
     <t>Ver</t>
   </si>
   <si>
     <t/>
-  </si>
-  <si>
-    <t>Squadra</t>
   </si>
 </sst>
 </file>
@@ -521,7 +518,7 @@
   <dimension ref="A1:U22"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="21" width="4" customWidth="1"/>
   </cols>
   <sheetData>
@@ -551,9 +548,6 @@
       <c r="U1" s="8"/>
     </row>
     <row r="2" spans="1:21">
-      <c r="A2" t="s">
-        <v>22</v>
-      </c>
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
@@ -623,61 +617,61 @@
         <v>21</v>
       </c>
       <c r="C3" s="4">
-        <v>9</v>
-      </c>
-      <c r="D3" s="5">
-        <v>6</v>
-      </c>
-      <c r="E3" s="5">
-        <v>8</v>
+        <v>12</v>
+      </c>
+      <c r="D3" s="4">
+        <v>10</v>
+      </c>
+      <c r="E3" s="4">
+        <v>13</v>
       </c>
       <c r="F3" s="5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G3" s="4">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H3" s="4">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="I3" s="4">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J3" s="4">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="K3" s="5">
-        <v>8</v>
-      </c>
-      <c r="L3" s="5">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="L3" s="4">
+        <v>11</v>
       </c>
       <c r="M3" s="4">
-        <v>9</v>
-      </c>
-      <c r="N3" s="4">
-        <v>13</v>
+        <v>11</v>
+      </c>
+      <c r="N3" s="5">
+        <v>2</v>
       </c>
       <c r="O3" s="5">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="P3" s="5">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q3" s="4">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="R3" s="5">
         <v>8</v>
       </c>
-      <c r="S3" s="4">
-        <v>10</v>
-      </c>
-      <c r="T3" s="4">
-        <v>11</v>
-      </c>
-      <c r="U3" s="4">
-        <v>9</v>
+      <c r="S3" s="5">
+        <v>4</v>
+      </c>
+      <c r="T3" s="5">
+        <v>7</v>
+      </c>
+      <c r="U3" s="5">
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:21">
@@ -685,7 +679,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="4">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>21</v>
@@ -694,16 +688,16 @@
         <v>8</v>
       </c>
       <c r="E4" s="5">
-        <v>6</v>
-      </c>
-      <c r="F4" s="4">
-        <v>10</v>
+        <v>7</v>
+      </c>
+      <c r="F4" s="5">
+        <v>8</v>
       </c>
       <c r="G4" s="4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H4" s="4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I4" s="5">
         <v>6</v>
@@ -712,45 +706,45 @@
         <v>9</v>
       </c>
       <c r="K4" s="4">
-        <v>10</v>
-      </c>
-      <c r="L4" s="5">
-        <v>7</v>
+        <v>9</v>
+      </c>
+      <c r="L4" s="4">
+        <v>12</v>
       </c>
       <c r="M4" s="4">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="N4" s="4">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="O4" s="4">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="P4" s="4">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="Q4" s="4">
-        <v>9</v>
-      </c>
-      <c r="R4" s="4">
-        <v>10</v>
+        <v>10</v>
+      </c>
+      <c r="R4" s="5">
+        <v>4</v>
       </c>
       <c r="S4" s="4">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="T4" s="5">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="U4" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:21">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="5">
-        <v>6</v>
+      <c r="B5" s="4">
+        <v>10</v>
       </c>
       <c r="C5" s="5">
         <v>8</v>
@@ -759,120 +753,120 @@
         <v>21</v>
       </c>
       <c r="E5" s="4">
-        <v>11</v>
-      </c>
-      <c r="F5" s="4">
-        <v>11</v>
-      </c>
-      <c r="G5" s="5">
-        <v>8</v>
-      </c>
-      <c r="H5" s="5">
-        <v>8</v>
-      </c>
-      <c r="I5" s="4">
-        <v>10</v>
+        <v>12</v>
+      </c>
+      <c r="F5" s="5">
+        <v>7</v>
+      </c>
+      <c r="G5" s="4">
+        <v>10</v>
+      </c>
+      <c r="H5" s="4">
+        <v>12</v>
+      </c>
+      <c r="I5" s="5">
+        <v>8</v>
       </c>
       <c r="J5" s="4">
-        <v>12</v>
-      </c>
-      <c r="K5" s="5">
-        <v>7</v>
-      </c>
-      <c r="L5" s="4">
-        <v>14</v>
+        <v>10</v>
+      </c>
+      <c r="K5" s="4">
+        <v>10</v>
+      </c>
+      <c r="L5" s="5">
+        <v>6</v>
       </c>
       <c r="M5" s="4">
-        <v>9</v>
-      </c>
-      <c r="N5" s="5">
-        <v>8</v>
+        <v>11</v>
+      </c>
+      <c r="N5" s="4">
+        <v>9</v>
       </c>
       <c r="O5" s="5">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="P5" s="4">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="Q5" s="4">
-        <v>12</v>
-      </c>
-      <c r="R5" s="5">
-        <v>7</v>
-      </c>
-      <c r="S5" s="5">
-        <v>5</v>
+        <v>9</v>
+      </c>
+      <c r="R5" s="4">
+        <v>9</v>
+      </c>
+      <c r="S5" s="4">
+        <v>9</v>
       </c>
       <c r="T5" s="5">
         <v>7</v>
       </c>
-      <c r="U5" s="4">
-        <v>10</v>
+      <c r="U5" s="5">
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:21">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="5">
-        <v>8</v>
+      <c r="B6" s="4">
+        <v>13</v>
       </c>
       <c r="C6" s="5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D6" s="4">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="4">
-        <v>13</v>
+      <c r="F6" s="5">
+        <v>6</v>
       </c>
       <c r="G6" s="5">
-        <v>6</v>
-      </c>
-      <c r="H6" s="5">
-        <v>6</v>
-      </c>
-      <c r="I6" s="5">
-        <v>8</v>
+        <v>7</v>
+      </c>
+      <c r="H6" s="4">
+        <v>13</v>
+      </c>
+      <c r="I6" s="4">
+        <v>12</v>
       </c>
       <c r="J6" s="4">
-        <v>9</v>
-      </c>
-      <c r="K6" s="4">
-        <v>12</v>
-      </c>
-      <c r="L6" s="4">
-        <v>10</v>
-      </c>
-      <c r="M6" s="4">
-        <v>11</v>
+        <v>13</v>
+      </c>
+      <c r="K6" s="5">
+        <v>5</v>
+      </c>
+      <c r="L6" s="5">
+        <v>7</v>
+      </c>
+      <c r="M6" s="5">
+        <v>7</v>
       </c>
       <c r="N6" s="5">
-        <v>2</v>
-      </c>
-      <c r="O6" s="4">
-        <v>11</v>
+        <v>4</v>
+      </c>
+      <c r="O6" s="5">
+        <v>8</v>
       </c>
       <c r="P6" s="4">
-        <v>9</v>
-      </c>
-      <c r="Q6" s="5">
-        <v>7</v>
+        <v>12</v>
+      </c>
+      <c r="Q6" s="4">
+        <v>14</v>
       </c>
       <c r="R6" s="4">
         <v>10</v>
       </c>
-      <c r="S6" s="4">
-        <v>9</v>
-      </c>
-      <c r="T6" s="4">
-        <v>12</v>
-      </c>
-      <c r="U6" s="4">
-        <v>11</v>
+      <c r="S6" s="5">
+        <v>6</v>
+      </c>
+      <c r="T6" s="5">
+        <v>8</v>
+      </c>
+      <c r="U6" s="5">
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:21">
@@ -880,64 +874,64 @@
         <v>5</v>
       </c>
       <c r="B7" s="5">
-        <v>5</v>
-      </c>
-      <c r="C7" s="4">
-        <v>10</v>
-      </c>
-      <c r="D7" s="4">
-        <v>11</v>
-      </c>
-      <c r="E7" s="4">
-        <v>13</v>
+        <v>3</v>
+      </c>
+      <c r="C7" s="5">
+        <v>8</v>
+      </c>
+      <c r="D7" s="5">
+        <v>7</v>
+      </c>
+      <c r="E7" s="5">
+        <v>6</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="G7" s="6">
-        <v>0</v>
-      </c>
-      <c r="H7" s="4">
-        <v>11</v>
-      </c>
-      <c r="I7" s="5">
-        <v>5</v>
+      <c r="G7" s="5">
+        <v>6</v>
+      </c>
+      <c r="H7" s="5">
+        <v>2</v>
+      </c>
+      <c r="I7" s="4">
+        <v>10</v>
       </c>
       <c r="J7" s="5">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K7" s="4">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="L7" s="4">
-        <v>11</v>
-      </c>
-      <c r="M7" s="4">
-        <v>14</v>
-      </c>
-      <c r="N7" s="5">
-        <v>6</v>
+        <v>9</v>
+      </c>
+      <c r="M7" s="5">
+        <v>8</v>
+      </c>
+      <c r="N7" s="4">
+        <v>15</v>
       </c>
       <c r="O7" s="4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="P7" s="4">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q7" s="5">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="R7" s="4">
-        <v>13</v>
-      </c>
-      <c r="S7" s="5">
-        <v>8</v>
+        <v>10</v>
+      </c>
+      <c r="S7" s="4">
+        <v>16</v>
       </c>
       <c r="T7" s="4">
-        <v>9</v>
-      </c>
-      <c r="U7" s="5">
-        <v>8</v>
+        <v>14</v>
+      </c>
+      <c r="U7" s="4">
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:21">
@@ -945,64 +939,64 @@
         <v>6</v>
       </c>
       <c r="B8" s="4">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C8" s="4">
-        <v>9</v>
-      </c>
-      <c r="D8" s="5">
-        <v>8</v>
+        <v>10</v>
+      </c>
+      <c r="D8" s="4">
+        <v>10</v>
       </c>
       <c r="E8" s="5">
-        <v>6</v>
-      </c>
-      <c r="F8" s="6">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="F8" s="5">
+        <v>6</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="H8" s="5">
-        <v>8</v>
-      </c>
-      <c r="I8" s="4">
-        <v>14</v>
+      <c r="H8" s="4">
+        <v>11</v>
+      </c>
+      <c r="I8" s="5">
+        <v>7</v>
       </c>
       <c r="J8" s="4">
-        <v>13</v>
-      </c>
-      <c r="K8" s="5">
-        <v>7</v>
-      </c>
-      <c r="L8" s="5">
-        <v>8</v>
-      </c>
-      <c r="M8" s="5">
-        <v>5</v>
+        <v>10</v>
+      </c>
+      <c r="K8" s="4">
+        <v>11</v>
+      </c>
+      <c r="L8" s="4">
+        <v>9</v>
+      </c>
+      <c r="M8" s="4">
+        <v>12</v>
       </c>
       <c r="N8" s="4">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="O8" s="4">
         <v>9</v>
       </c>
       <c r="P8" s="5">
-        <v>7</v>
-      </c>
-      <c r="Q8" s="4">
-        <v>12</v>
-      </c>
-      <c r="R8" s="5">
-        <v>6</v>
+        <v>1</v>
+      </c>
+      <c r="Q8" s="5">
+        <v>8</v>
+      </c>
+      <c r="R8" s="4">
+        <v>9</v>
       </c>
       <c r="S8" s="4">
-        <v>11</v>
-      </c>
-      <c r="T8" s="4">
-        <v>10</v>
+        <v>9</v>
+      </c>
+      <c r="T8" s="5">
+        <v>7</v>
       </c>
       <c r="U8" s="4">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:21">
@@ -1010,61 +1004,61 @@
         <v>7</v>
       </c>
       <c r="B9" s="4">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C9" s="4">
-        <v>10</v>
-      </c>
-      <c r="D9" s="5">
-        <v>8</v>
-      </c>
-      <c r="E9" s="5">
-        <v>6</v>
-      </c>
-      <c r="F9" s="4">
-        <v>11</v>
-      </c>
-      <c r="G9" s="5">
-        <v>8</v>
+        <v>11</v>
+      </c>
+      <c r="D9" s="4">
+        <v>12</v>
+      </c>
+      <c r="E9" s="4">
+        <v>13</v>
+      </c>
+      <c r="F9" s="5">
+        <v>2</v>
+      </c>
+      <c r="G9" s="4">
+        <v>11</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="I9" s="5">
-        <v>6</v>
+      <c r="I9" s="4">
+        <v>9</v>
       </c>
       <c r="J9" s="4">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="K9" s="5">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L9" s="4">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M9" s="4">
-        <v>13</v>
-      </c>
-      <c r="N9" s="4">
-        <v>12</v>
+        <v>11</v>
+      </c>
+      <c r="N9" s="5">
+        <v>4</v>
       </c>
       <c r="O9" s="5">
-        <v>7</v>
-      </c>
-      <c r="P9" s="4">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="P9" s="5">
+        <v>7</v>
       </c>
       <c r="Q9" s="4">
-        <v>12</v>
-      </c>
-      <c r="R9" s="4">
-        <v>10</v>
+        <v>14</v>
+      </c>
+      <c r="R9" s="5">
+        <v>8</v>
       </c>
       <c r="S9" s="5">
-        <v>7</v>
-      </c>
-      <c r="T9" s="4">
-        <v>10</v>
+        <v>5</v>
+      </c>
+      <c r="T9" s="5">
+        <v>4</v>
       </c>
       <c r="U9" s="5">
         <v>6</v>
@@ -1075,64 +1069,64 @@
         <v>8</v>
       </c>
       <c r="B10" s="4">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C10" s="5">
         <v>6</v>
       </c>
-      <c r="D10" s="4">
-        <v>10</v>
-      </c>
-      <c r="E10" s="5">
-        <v>8</v>
-      </c>
-      <c r="F10" s="5">
-        <v>5</v>
-      </c>
-      <c r="G10" s="4">
-        <v>14</v>
-      </c>
-      <c r="H10" s="5">
-        <v>6</v>
+      <c r="D10" s="5">
+        <v>8</v>
+      </c>
+      <c r="E10" s="4">
+        <v>12</v>
+      </c>
+      <c r="F10" s="4">
+        <v>10</v>
+      </c>
+      <c r="G10" s="5">
+        <v>7</v>
+      </c>
+      <c r="H10" s="4">
+        <v>9</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>21</v>
       </c>
       <c r="J10" s="4">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K10" s="4">
-        <v>9</v>
-      </c>
-      <c r="L10" s="4">
-        <v>11</v>
-      </c>
-      <c r="M10" s="6">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="L10" s="5">
+        <v>8</v>
+      </c>
+      <c r="M10" s="5">
+        <v>1</v>
       </c>
       <c r="N10" s="4">
-        <v>11</v>
-      </c>
-      <c r="O10" s="4">
-        <v>11</v>
-      </c>
-      <c r="P10" s="5">
-        <v>8</v>
+        <v>10</v>
+      </c>
+      <c r="O10" s="5">
+        <v>5</v>
+      </c>
+      <c r="P10" s="4">
+        <v>11</v>
       </c>
       <c r="Q10" s="4">
-        <v>10</v>
-      </c>
-      <c r="R10" s="5">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="R10" s="4">
+        <v>12</v>
       </c>
       <c r="S10" s="5">
         <v>7</v>
       </c>
       <c r="T10" s="4">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="U10" s="4">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:21">
@@ -1140,64 +1134,64 @@
         <v>9</v>
       </c>
       <c r="B11" s="4">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C11" s="4">
         <v>9</v>
       </c>
       <c r="D11" s="4">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E11" s="4">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F11" s="5">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G11" s="4">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H11" s="4">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="I11" s="4">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J11" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="K11" s="4">
-        <v>10</v>
+      <c r="K11" s="5">
+        <v>5</v>
       </c>
       <c r="L11" s="4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M11" s="5">
         <v>8</v>
       </c>
       <c r="N11" s="5">
-        <v>8</v>
-      </c>
-      <c r="O11" s="4">
-        <v>9</v>
-      </c>
-      <c r="P11" s="5">
-        <v>8</v>
+        <v>5</v>
+      </c>
+      <c r="O11" s="5">
+        <v>5</v>
+      </c>
+      <c r="P11" s="4">
+        <v>9</v>
       </c>
       <c r="Q11" s="4">
-        <v>9</v>
-      </c>
-      <c r="R11" s="6">
+        <v>14</v>
+      </c>
+      <c r="R11" s="4">
+        <v>12</v>
+      </c>
+      <c r="S11" s="6">
         <v>0</v>
       </c>
-      <c r="S11" s="4">
-        <v>9</v>
-      </c>
-      <c r="T11" s="4">
-        <v>9</v>
+      <c r="T11" s="5">
+        <v>7</v>
       </c>
       <c r="U11" s="4">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:21">
@@ -1205,31 +1199,31 @@
         <v>10</v>
       </c>
       <c r="B12" s="5">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C12" s="4">
-        <v>10</v>
-      </c>
-      <c r="D12" s="5">
-        <v>7</v>
-      </c>
-      <c r="E12" s="4">
-        <v>12</v>
+        <v>9</v>
+      </c>
+      <c r="D12" s="4">
+        <v>10</v>
+      </c>
+      <c r="E12" s="5">
+        <v>5</v>
       </c>
       <c r="F12" s="4">
-        <v>12</v>
-      </c>
-      <c r="G12" s="5">
-        <v>7</v>
+        <v>14</v>
+      </c>
+      <c r="G12" s="4">
+        <v>11</v>
       </c>
       <c r="H12" s="5">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I12" s="4">
-        <v>9</v>
-      </c>
-      <c r="J12" s="4">
-        <v>10</v>
+        <v>10</v>
+      </c>
+      <c r="J12" s="5">
+        <v>5</v>
       </c>
       <c r="K12" s="3" t="s">
         <v>21</v>
@@ -1237,17 +1231,17 @@
       <c r="L12" s="5">
         <v>7</v>
       </c>
-      <c r="M12" s="4">
-        <v>10</v>
-      </c>
-      <c r="N12" s="5">
-        <v>6</v>
+      <c r="M12" s="5">
+        <v>8</v>
+      </c>
+      <c r="N12" s="4">
+        <v>18</v>
       </c>
       <c r="O12" s="4">
-        <v>15</v>
-      </c>
-      <c r="P12" s="4">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="P12" s="5">
+        <v>8</v>
       </c>
       <c r="Q12" s="6">
         <v>0</v>
@@ -1256,45 +1250,45 @@
         <v>9</v>
       </c>
       <c r="S12" s="4">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="T12" s="4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="U12" s="4">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:21">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="5">
-        <v>6</v>
-      </c>
-      <c r="C13" s="5">
-        <v>7</v>
-      </c>
-      <c r="D13" s="4">
-        <v>14</v>
-      </c>
-      <c r="E13" s="4">
-        <v>10</v>
+      <c r="B13" s="4">
+        <v>11</v>
+      </c>
+      <c r="C13" s="4">
+        <v>12</v>
+      </c>
+      <c r="D13" s="5">
+        <v>6</v>
+      </c>
+      <c r="E13" s="5">
+        <v>7</v>
       </c>
       <c r="F13" s="4">
-        <v>11</v>
-      </c>
-      <c r="G13" s="5">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="G13" s="4">
+        <v>9</v>
       </c>
       <c r="H13" s="4">
-        <v>11</v>
-      </c>
-      <c r="I13" s="4">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="I13" s="5">
+        <v>8</v>
       </c>
       <c r="J13" s="4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K13" s="5">
         <v>7</v>
@@ -1302,32 +1296,32 @@
       <c r="L13" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="M13" s="5">
-        <v>8</v>
+      <c r="M13" s="4">
+        <v>11</v>
       </c>
       <c r="N13" s="5">
         <v>8</v>
       </c>
-      <c r="O13" s="5">
-        <v>5</v>
+      <c r="O13" s="4">
+        <v>9</v>
       </c>
       <c r="P13" s="4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q13" s="4">
         <v>12</v>
       </c>
-      <c r="R13" s="4">
-        <v>9</v>
+      <c r="R13" s="5">
+        <v>7</v>
       </c>
       <c r="S13" s="5">
-        <v>4</v>
-      </c>
-      <c r="T13" s="4">
-        <v>11</v>
-      </c>
-      <c r="U13" s="4">
-        <v>10</v>
+        <v>8</v>
+      </c>
+      <c r="T13" s="5">
+        <v>6</v>
+      </c>
+      <c r="U13" s="5">
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:21">
@@ -1335,37 +1329,37 @@
         <v>12</v>
       </c>
       <c r="B14" s="4">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C14" s="4">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D14" s="4">
-        <v>9</v>
-      </c>
-      <c r="E14" s="4">
-        <v>11</v>
-      </c>
-      <c r="F14" s="4">
-        <v>14</v>
-      </c>
-      <c r="G14" s="5">
-        <v>5</v>
+        <v>11</v>
+      </c>
+      <c r="E14" s="5">
+        <v>7</v>
+      </c>
+      <c r="F14" s="5">
+        <v>8</v>
+      </c>
+      <c r="G14" s="4">
+        <v>12</v>
       </c>
       <c r="H14" s="4">
-        <v>13</v>
-      </c>
-      <c r="I14" s="6">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="I14" s="5">
+        <v>1</v>
       </c>
       <c r="J14" s="5">
         <v>8</v>
       </c>
-      <c r="K14" s="4">
-        <v>10</v>
-      </c>
-      <c r="L14" s="5">
-        <v>8</v>
+      <c r="K14" s="5">
+        <v>8</v>
+      </c>
+      <c r="L14" s="4">
+        <v>11</v>
       </c>
       <c r="M14" s="3" t="s">
         <v>21</v>
@@ -1373,61 +1367,61 @@
       <c r="N14" s="5">
         <v>8</v>
       </c>
-      <c r="O14" s="5">
-        <v>8</v>
-      </c>
-      <c r="P14" s="4">
-        <v>11</v>
+      <c r="O14" s="4">
+        <v>13</v>
+      </c>
+      <c r="P14" s="5">
+        <v>7</v>
       </c>
       <c r="Q14" s="4">
-        <v>9</v>
-      </c>
-      <c r="R14" s="4">
-        <v>11</v>
+        <v>11</v>
+      </c>
+      <c r="R14" s="5">
+        <v>8</v>
       </c>
       <c r="S14" s="4">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="T14" s="5">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="U14" s="5">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:21">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="4">
-        <v>13</v>
+      <c r="B15" s="5">
+        <v>2</v>
       </c>
       <c r="C15" s="4">
-        <v>11</v>
-      </c>
-      <c r="D15" s="5">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="D15" s="4">
+        <v>9</v>
       </c>
       <c r="E15" s="5">
-        <v>2</v>
-      </c>
-      <c r="F15" s="5">
-        <v>6</v>
+        <v>4</v>
+      </c>
+      <c r="F15" s="4">
+        <v>15</v>
       </c>
       <c r="G15" s="4">
-        <v>13</v>
-      </c>
-      <c r="H15" s="4">
-        <v>12</v>
+        <v>10</v>
+      </c>
+      <c r="H15" s="5">
+        <v>4</v>
       </c>
       <c r="I15" s="4">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J15" s="5">
-        <v>8</v>
-      </c>
-      <c r="K15" s="5">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="K15" s="4">
+        <v>18</v>
       </c>
       <c r="L15" s="5">
         <v>8</v>
@@ -1438,26 +1432,26 @@
       <c r="N15" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="O15" s="5">
-        <v>7</v>
+      <c r="O15" s="4">
+        <v>11</v>
       </c>
       <c r="P15" s="4">
-        <v>10</v>
-      </c>
-      <c r="Q15" s="4">
-        <v>13</v>
+        <v>9</v>
+      </c>
+      <c r="Q15" s="5">
+        <v>1</v>
       </c>
       <c r="R15" s="4">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="S15" s="4">
-        <v>9</v>
-      </c>
-      <c r="T15" s="5">
-        <v>7</v>
-      </c>
-      <c r="U15" s="5">
-        <v>8</v>
+        <v>14</v>
+      </c>
+      <c r="T15" s="4">
+        <v>12</v>
+      </c>
+      <c r="U15" s="4">
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:21">
@@ -1465,64 +1459,64 @@
         <v>14</v>
       </c>
       <c r="B16" s="5">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C16" s="4">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D16" s="5">
-        <v>5</v>
-      </c>
-      <c r="E16" s="4">
-        <v>11</v>
+        <v>8</v>
+      </c>
+      <c r="E16" s="5">
+        <v>8</v>
       </c>
       <c r="F16" s="4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G16" s="4">
         <v>9</v>
       </c>
       <c r="H16" s="5">
-        <v>7</v>
-      </c>
-      <c r="I16" s="4">
-        <v>11</v>
-      </c>
-      <c r="J16" s="4">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="I16" s="5">
+        <v>5</v>
+      </c>
+      <c r="J16" s="5">
+        <v>5</v>
       </c>
       <c r="K16" s="4">
-        <v>15</v>
-      </c>
-      <c r="L16" s="5">
-        <v>5</v>
-      </c>
-      <c r="M16" s="5">
-        <v>8</v>
-      </c>
-      <c r="N16" s="5">
-        <v>7</v>
+        <v>11</v>
+      </c>
+      <c r="L16" s="4">
+        <v>9</v>
+      </c>
+      <c r="M16" s="4">
+        <v>13</v>
+      </c>
+      <c r="N16" s="4">
+        <v>11</v>
       </c>
       <c r="O16" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="P16" s="5">
-        <v>7</v>
+      <c r="P16" s="4">
+        <v>10</v>
       </c>
       <c r="Q16" s="5">
-        <v>4</v>
-      </c>
-      <c r="R16" s="4">
-        <v>10</v>
+        <v>8</v>
+      </c>
+      <c r="R16" s="5">
+        <v>5</v>
       </c>
       <c r="S16" s="4">
         <v>14</v>
       </c>
       <c r="T16" s="4">
-        <v>11</v>
-      </c>
-      <c r="U16" s="4">
-        <v>11</v>
+        <v>9</v>
+      </c>
+      <c r="U16" s="5">
+        <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:21">
@@ -1530,64 +1524,64 @@
         <v>15</v>
       </c>
       <c r="B17" s="5">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C17" s="4">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D17" s="4">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E17" s="4">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F17" s="4">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G17" s="5">
-        <v>7</v>
-      </c>
-      <c r="H17" s="4">
-        <v>9</v>
-      </c>
-      <c r="I17" s="5">
-        <v>8</v>
-      </c>
-      <c r="J17" s="5">
-        <v>8</v>
-      </c>
-      <c r="K17" s="4">
-        <v>9</v>
+        <v>1</v>
+      </c>
+      <c r="H17" s="5">
+        <v>7</v>
+      </c>
+      <c r="I17" s="4">
+        <v>11</v>
+      </c>
+      <c r="J17" s="4">
+        <v>9</v>
+      </c>
+      <c r="K17" s="5">
+        <v>8</v>
       </c>
       <c r="L17" s="4">
-        <v>9</v>
-      </c>
-      <c r="M17" s="4">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="M17" s="5">
+        <v>7</v>
       </c>
       <c r="N17" s="4">
-        <v>10</v>
-      </c>
-      <c r="O17" s="5">
-        <v>7</v>
+        <v>9</v>
+      </c>
+      <c r="O17" s="4">
+        <v>10</v>
       </c>
       <c r="P17" s="3" t="s">
         <v>21</v>
       </c>
       <c r="Q17" s="4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R17" s="4">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="S17" s="4">
-        <v>9</v>
-      </c>
-      <c r="T17" s="5">
-        <v>2</v>
+        <v>10</v>
+      </c>
+      <c r="T17" s="4">
+        <v>11</v>
       </c>
       <c r="U17" s="5">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:21">
@@ -1595,31 +1589,31 @@
         <v>16</v>
       </c>
       <c r="B18" s="4">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C18" s="4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D18" s="4">
-        <v>12</v>
-      </c>
-      <c r="E18" s="5">
-        <v>7</v>
+        <v>9</v>
+      </c>
+      <c r="E18" s="4">
+        <v>14</v>
       </c>
       <c r="F18" s="5">
-        <v>7</v>
-      </c>
-      <c r="G18" s="4">
-        <v>12</v>
+        <v>5</v>
+      </c>
+      <c r="G18" s="5">
+        <v>8</v>
       </c>
       <c r="H18" s="4">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="I18" s="4">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J18" s="4">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="K18" s="6">
         <v>0</v>
@@ -1628,16 +1622,16 @@
         <v>12</v>
       </c>
       <c r="M18" s="4">
-        <v>9</v>
-      </c>
-      <c r="N18" s="4">
-        <v>13</v>
+        <v>11</v>
+      </c>
+      <c r="N18" s="5">
+        <v>1</v>
       </c>
       <c r="O18" s="5">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="P18" s="4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q18" s="3" t="s">
         <v>21</v>
@@ -1646,13 +1640,13 @@
         <v>10</v>
       </c>
       <c r="S18" s="5">
-        <v>6</v>
-      </c>
-      <c r="T18" s="4">
-        <v>9</v>
-      </c>
-      <c r="U18" s="4">
-        <v>9</v>
+        <v>5</v>
+      </c>
+      <c r="T18" s="5">
+        <v>8</v>
+      </c>
+      <c r="U18" s="5">
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:21">
@@ -1662,47 +1656,47 @@
       <c r="B19" s="5">
         <v>8</v>
       </c>
-      <c r="C19" s="4">
-        <v>10</v>
-      </c>
-      <c r="D19" s="5">
-        <v>7</v>
+      <c r="C19" s="5">
+        <v>4</v>
+      </c>
+      <c r="D19" s="4">
+        <v>9</v>
       </c>
       <c r="E19" s="4">
         <v>10</v>
       </c>
       <c r="F19" s="4">
-        <v>13</v>
-      </c>
-      <c r="G19" s="5">
-        <v>6</v>
-      </c>
-      <c r="H19" s="4">
-        <v>10</v>
-      </c>
-      <c r="I19" s="5">
-        <v>8</v>
-      </c>
-      <c r="J19" s="6">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="G19" s="4">
+        <v>9</v>
+      </c>
+      <c r="H19" s="5">
+        <v>8</v>
+      </c>
+      <c r="I19" s="4">
+        <v>12</v>
+      </c>
+      <c r="J19" s="4">
+        <v>12</v>
       </c>
       <c r="K19" s="4">
         <v>9</v>
       </c>
-      <c r="L19" s="4">
-        <v>9</v>
-      </c>
-      <c r="M19" s="4">
-        <v>11</v>
+      <c r="L19" s="5">
+        <v>7</v>
+      </c>
+      <c r="M19" s="5">
+        <v>8</v>
       </c>
       <c r="N19" s="4">
-        <v>11</v>
-      </c>
-      <c r="O19" s="4">
-        <v>10</v>
+        <v>9</v>
+      </c>
+      <c r="O19" s="5">
+        <v>5</v>
       </c>
       <c r="P19" s="4">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="Q19" s="4">
         <v>10</v>
@@ -1710,206 +1704,206 @@
       <c r="R19" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="S19" s="4">
-        <v>10</v>
+      <c r="S19" s="5">
+        <v>7</v>
       </c>
       <c r="T19" s="4">
-        <v>10</v>
-      </c>
-      <c r="U19" s="5">
-        <v>8</v>
+        <v>11</v>
+      </c>
+      <c r="U19" s="4">
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:21">
       <c r="A20" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="4">
-        <v>10</v>
+      <c r="B20" s="5">
+        <v>4</v>
       </c>
       <c r="C20" s="4">
-        <v>14</v>
-      </c>
-      <c r="D20" s="5">
-        <v>5</v>
-      </c>
-      <c r="E20" s="4">
-        <v>9</v>
-      </c>
-      <c r="F20" s="5">
-        <v>8</v>
+        <v>10</v>
+      </c>
+      <c r="D20" s="4">
+        <v>9</v>
+      </c>
+      <c r="E20" s="5">
+        <v>6</v>
+      </c>
+      <c r="F20" s="4">
+        <v>16</v>
       </c>
       <c r="G20" s="4">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="H20" s="5">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I20" s="5">
         <v>7</v>
       </c>
-      <c r="J20" s="4">
-        <v>9</v>
+      <c r="J20" s="6">
+        <v>0</v>
       </c>
       <c r="K20" s="4">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="L20" s="5">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M20" s="4">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="N20" s="4">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="O20" s="4">
         <v>14</v>
       </c>
       <c r="P20" s="4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q20" s="5">
-        <v>6</v>
-      </c>
-      <c r="R20" s="4">
-        <v>10</v>
+        <v>5</v>
+      </c>
+      <c r="R20" s="5">
+        <v>7</v>
       </c>
       <c r="S20" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="T20" s="5">
-        <v>8</v>
-      </c>
-      <c r="U20" s="5">
-        <v>6</v>
+      <c r="T20" s="4">
+        <v>12</v>
+      </c>
+      <c r="U20" s="4">
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:21">
       <c r="A21" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="4">
-        <v>11</v>
+      <c r="B21" s="5">
+        <v>7</v>
       </c>
       <c r="C21" s="5">
+        <v>7</v>
+      </c>
+      <c r="D21" s="5">
+        <v>7</v>
+      </c>
+      <c r="E21" s="5">
+        <v>8</v>
+      </c>
+      <c r="F21" s="4">
+        <v>14</v>
+      </c>
+      <c r="G21" s="5">
+        <v>7</v>
+      </c>
+      <c r="H21" s="5">
         <v>4</v>
       </c>
-      <c r="D21" s="5">
-        <v>7</v>
-      </c>
-      <c r="E21" s="4">
-        <v>12</v>
-      </c>
-      <c r="F21" s="4">
-        <v>9</v>
-      </c>
-      <c r="G21" s="4">
-        <v>10</v>
-      </c>
-      <c r="H21" s="4">
-        <v>10</v>
-      </c>
       <c r="I21" s="4">
-        <v>11</v>
-      </c>
-      <c r="J21" s="4">
-        <v>9</v>
+        <v>13</v>
+      </c>
+      <c r="J21" s="5">
+        <v>7</v>
       </c>
       <c r="K21" s="4">
-        <v>10</v>
-      </c>
-      <c r="L21" s="4">
-        <v>11</v>
+        <v>11</v>
+      </c>
+      <c r="L21" s="5">
+        <v>6</v>
       </c>
       <c r="M21" s="5">
-        <v>8</v>
-      </c>
-      <c r="N21" s="5">
-        <v>7</v>
+        <v>6</v>
+      </c>
+      <c r="N21" s="4">
+        <v>12</v>
       </c>
       <c r="O21" s="4">
-        <v>11</v>
-      </c>
-      <c r="P21" s="5">
-        <v>2</v>
-      </c>
-      <c r="Q21" s="4">
-        <v>9</v>
+        <v>9</v>
+      </c>
+      <c r="P21" s="4">
+        <v>11</v>
+      </c>
+      <c r="Q21" s="5">
+        <v>8</v>
       </c>
       <c r="R21" s="4">
-        <v>10</v>
-      </c>
-      <c r="S21" s="5">
-        <v>8</v>
+        <v>11</v>
+      </c>
+      <c r="S21" s="4">
+        <v>12</v>
       </c>
       <c r="T21" s="3" t="s">
         <v>21</v>
       </c>
       <c r="U21" s="4">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="22" spans="1:21">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="4">
-        <v>9</v>
+      <c r="B22" s="5">
+        <v>6</v>
       </c>
       <c r="C22" s="5">
-        <v>4</v>
-      </c>
-      <c r="D22" s="4">
-        <v>10</v>
-      </c>
-      <c r="E22" s="4">
-        <v>11</v>
-      </c>
-      <c r="F22" s="5">
-        <v>8</v>
+        <v>5</v>
+      </c>
+      <c r="D22" s="5">
+        <v>7</v>
+      </c>
+      <c r="E22" s="5">
+        <v>7</v>
+      </c>
+      <c r="F22" s="4">
+        <v>11</v>
       </c>
       <c r="G22" s="4">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H22" s="5">
         <v>6</v>
       </c>
       <c r="I22" s="4">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="J22" s="4">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="K22" s="4">
-        <v>10</v>
-      </c>
-      <c r="L22" s="4">
-        <v>10</v>
+        <v>13</v>
+      </c>
+      <c r="L22" s="5">
+        <v>8</v>
       </c>
       <c r="M22" s="5">
-        <v>4</v>
-      </c>
-      <c r="N22" s="5">
-        <v>8</v>
-      </c>
-      <c r="O22" s="4">
-        <v>11</v>
+        <v>7</v>
+      </c>
+      <c r="N22" s="4">
+        <v>13</v>
+      </c>
+      <c r="O22" s="5">
+        <v>7</v>
       </c>
       <c r="P22" s="5">
-        <v>8</v>
-      </c>
-      <c r="Q22" s="4">
-        <v>9</v>
-      </c>
-      <c r="R22" s="5">
-        <v>8</v>
-      </c>
-      <c r="S22" s="5">
-        <v>6</v>
+        <v>6</v>
+      </c>
+      <c r="Q22" s="5">
+        <v>6</v>
+      </c>
+      <c r="R22" s="4">
+        <v>13</v>
+      </c>
+      <c r="S22" s="4">
+        <v>10</v>
       </c>
       <c r="T22" s="4">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="U22" s="3" t="s">
         <v>21</v>

</xml_diff>